<commit_message>
Fix discounting: dismissal and mortality use mid-year (t-0.5), resignation and retirement use end-of-year per IAS 19 formula
</commit_message>
<xml_diff>
--- a/output/results_ias19.xlsx
+++ b/output/results_ias19.xlsx
@@ -691,7 +691,7 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>22423.41</v>
+        <v>22426.06</v>
       </c>
     </row>
     <row r="4">
@@ -777,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>712621.1800000001</v>
+        <v>713509.48</v>
       </c>
     </row>
     <row r="5">
@@ -857,7 +857,7 @@
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>209636.27</v>
+        <v>208693.77</v>
       </c>
     </row>
     <row r="6">
@@ -1019,7 +1019,7 @@
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>427418.73</v>
+        <v>428247.3</v>
       </c>
     </row>
     <row r="8">
@@ -1175,7 +1175,7 @@
         <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>300241.69</v>
+        <v>299563.55</v>
       </c>
     </row>
     <row r="10">
@@ -1327,7 +1327,7 @@
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>12622.37</v>
+        <v>12625.51</v>
       </c>
     </row>
     <row r="12">
@@ -1407,7 +1407,7 @@
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>456061.81</v>
+        <v>457374.31</v>
       </c>
     </row>
     <row r="13">
@@ -1559,7 +1559,7 @@
         <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>359432.01</v>
+        <v>360564.23</v>
       </c>
     </row>
     <row r="15">
@@ -1645,7 +1645,7 @@
         <v>1</v>
       </c>
       <c r="X15" t="n">
-        <v>455808.28</v>
+        <v>454623.95</v>
       </c>
     </row>
     <row r="16">
@@ -1727,7 +1727,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>85539.06</v>
+        <v>85559.59</v>
       </c>
     </row>
     <row r="17">
@@ -1891,7 +1891,7 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>67489.71000000001</v>
+        <v>67635.50999999999</v>
       </c>
     </row>
     <row r="19">
@@ -2129,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>149691.82</v>
+        <v>149137</v>
       </c>
     </row>
     <row r="22">
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>313338.33</v>
+        <v>314033.59</v>
       </c>
     </row>
     <row r="24">
@@ -2369,7 +2369,7 @@
         <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>48263.26</v>
+        <v>48393.6</v>
       </c>
     </row>
     <row r="25">
@@ -2741,7 +2741,7 @@
         <v>1</v>
       </c>
       <c r="X29" t="n">
-        <v>327742.32</v>
+        <v>326065.99</v>
       </c>
     </row>
     <row r="30">
@@ -3037,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="X33" t="n">
-        <v>214666.05</v>
+        <v>215746.67</v>
       </c>
     </row>
     <row r="34">
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>101070.27</v>
+        <v>100508.01</v>
       </c>
     </row>
     <row r="35">
@@ -3199,7 +3199,7 @@
         <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>308574.42</v>
+        <v>309931.97</v>
       </c>
     </row>
     <row r="36">
@@ -3427,7 +3427,7 @@
         <v>0</v>
       </c>
       <c r="X38" t="n">
-        <v>173783.49</v>
+        <v>174364.96</v>
       </c>
     </row>
     <row r="39">
@@ -3509,7 +3509,7 @@
         <v>0</v>
       </c>
       <c r="X39" t="n">
-        <v>23197.17</v>
+        <v>23202.17</v>
       </c>
     </row>
     <row r="40">
@@ -3737,7 +3737,7 @@
         <v>0</v>
       </c>
       <c r="X42" t="n">
-        <v>160749.29</v>
+        <v>160941.53</v>
       </c>
     </row>
     <row r="43">
@@ -3959,7 +3959,7 @@
         <v>0</v>
       </c>
       <c r="X45" t="n">
-        <v>22319.89</v>
+        <v>22324.89</v>
       </c>
     </row>
     <row r="46">
@@ -4041,7 +4041,7 @@
         <v>0</v>
       </c>
       <c r="X46" t="n">
-        <v>5783.67</v>
+        <v>5783.71</v>
       </c>
     </row>
     <row r="47">
@@ -4121,7 +4121,7 @@
         <v>1</v>
       </c>
       <c r="X47" t="n">
-        <v>408829.16</v>
+        <v>408132.69</v>
       </c>
     </row>
     <row r="48">
@@ -4203,7 +4203,7 @@
         <v>0</v>
       </c>
       <c r="X48" t="n">
-        <v>27671.31</v>
+        <v>27708.4</v>
       </c>
     </row>
     <row r="49">
@@ -4373,7 +4373,7 @@
         <v>0</v>
       </c>
       <c r="X50" t="n">
-        <v>86991.61</v>
+        <v>87009.78999999999</v>
       </c>
     </row>
     <row r="51">
@@ -4531,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="X52" t="n">
-        <v>28568.9</v>
+        <v>28675.26</v>
       </c>
     </row>
     <row r="53">
@@ -4921,7 +4921,7 @@
         <v>0</v>
       </c>
       <c r="X57" t="n">
-        <v>308029.3</v>
+        <v>309447.18</v>
       </c>
     </row>
     <row r="58">
@@ -5323,7 +5323,7 @@
         <v>0</v>
       </c>
       <c r="X62" t="n">
-        <v>187417.87</v>
+        <v>188041.9</v>
       </c>
     </row>
     <row r="63">
@@ -5561,7 +5561,7 @@
         <v>1</v>
       </c>
       <c r="X65" t="n">
-        <v>402614.18</v>
+        <v>401217.09</v>
       </c>
     </row>
     <row r="66">
@@ -5647,7 +5647,7 @@
         <v>0</v>
       </c>
       <c r="X66" t="n">
-        <v>457108.74</v>
+        <v>458157.58</v>
       </c>
     </row>
     <row r="67">
@@ -5809,7 +5809,7 @@
         <v>1</v>
       </c>
       <c r="X68" t="n">
-        <v>131862.55</v>
+        <v>131325.07</v>
       </c>
     </row>
     <row r="69">
@@ -5897,7 +5897,7 @@
         <v>0</v>
       </c>
       <c r="X69" t="n">
-        <v>69434.73</v>
+        <v>69452.21000000001</v>
       </c>
     </row>
     <row r="70">
@@ -5983,7 +5983,7 @@
         <v>1</v>
       </c>
       <c r="X70" t="n">
-        <v>356071.74</v>
+        <v>355341.73</v>
       </c>
     </row>
     <row r="71">
@@ -6141,7 +6141,7 @@
         <v>0</v>
       </c>
       <c r="X72" t="n">
-        <v>46099.15</v>
+        <v>46110.78</v>
       </c>
     </row>
     <row r="73">
@@ -6221,7 +6221,7 @@
         <v>1</v>
       </c>
       <c r="X73" t="n">
-        <v>659845.97</v>
+        <v>657606.2</v>
       </c>
     </row>
     <row r="74">
@@ -6303,7 +6303,7 @@
         <v>0</v>
       </c>
       <c r="X74" t="n">
-        <v>181007.42</v>
+        <v>181365.03</v>
       </c>
     </row>
     <row r="75">
@@ -6383,7 +6383,7 @@
         <v>1</v>
       </c>
       <c r="X75" t="n">
-        <v>324049.26</v>
+        <v>322927.82</v>
       </c>
     </row>
     <row r="76">
@@ -6463,7 +6463,7 @@
         <v>1</v>
       </c>
       <c r="X76" t="n">
-        <v>278422.85</v>
+        <v>277403.2</v>
       </c>
     </row>
     <row r="77">
@@ -6543,7 +6543,7 @@
         <v>0</v>
       </c>
       <c r="X77" t="n">
-        <v>288015.75</v>
+        <v>288901.99</v>
       </c>
     </row>
     <row r="78">
@@ -6771,7 +6771,7 @@
         <v>0</v>
       </c>
       <c r="X80" t="n">
-        <v>24460.57</v>
+        <v>24507.25</v>
       </c>
     </row>
     <row r="81">
@@ -7233,7 +7233,7 @@
         <v>0</v>
       </c>
       <c r="X86" t="n">
-        <v>38098.97</v>
+        <v>38207.49</v>
       </c>
     </row>
     <row r="87">
@@ -7385,7 +7385,7 @@
         <v>0</v>
       </c>
       <c r="X88" t="n">
-        <v>54837.48</v>
+        <v>54847.65</v>
       </c>
     </row>
     <row r="89">
@@ -7467,7 +7467,7 @@
         <v>0</v>
       </c>
       <c r="X89" t="n">
-        <v>50915.73</v>
+        <v>50924.92</v>
       </c>
     </row>
     <row r="90">
@@ -7553,7 +7553,7 @@
         <v>0</v>
       </c>
       <c r="X90" t="n">
-        <v>431973.67</v>
+        <v>433683.23</v>
       </c>
     </row>
     <row r="91">
@@ -7635,7 +7635,7 @@
         <v>0</v>
       </c>
       <c r="X91" t="n">
-        <v>87518.27</v>
+        <v>87880.08</v>
       </c>
     </row>
     <row r="92">
@@ -7715,7 +7715,7 @@
         <v>1</v>
       </c>
       <c r="X92" t="n">
-        <v>118347.95</v>
+        <v>117680.51</v>
       </c>
     </row>
     <row r="93">
@@ -7935,7 +7935,7 @@
         <v>1</v>
       </c>
       <c r="X95" t="n">
-        <v>232412.11</v>
+        <v>231185.01</v>
       </c>
     </row>
     <row r="96">
@@ -8087,7 +8087,7 @@
         <v>0</v>
       </c>
       <c r="X97" t="n">
-        <v>18070.78</v>
+        <v>18074.03</v>
       </c>
     </row>
     <row r="98">
@@ -8169,7 +8169,7 @@
         <v>0</v>
       </c>
       <c r="X98" t="n">
-        <v>14187.04</v>
+        <v>14189.58</v>
       </c>
     </row>
     <row r="99">
@@ -8249,7 +8249,7 @@
         <v>1</v>
       </c>
       <c r="X99" t="n">
-        <v>199436.65</v>
+        <v>198695.91</v>
       </c>
     </row>
     <row r="100">
@@ -8329,7 +8329,7 @@
         <v>1</v>
       </c>
       <c r="X100" t="n">
-        <v>394006.13</v>
+        <v>392498.4</v>
       </c>
     </row>
     <row r="101">
@@ -8563,7 +8563,7 @@
         <v>0</v>
       </c>
       <c r="X103" t="n">
-        <v>17135.86</v>
+        <v>17137.4</v>
       </c>
     </row>
     <row r="104">
@@ -8645,7 +8645,7 @@
         <v>0</v>
       </c>
       <c r="X104" t="n">
-        <v>21443.47</v>
+        <v>21445</v>
       </c>
     </row>
     <row r="105">
@@ -8867,7 +8867,7 @@
         <v>0</v>
       </c>
       <c r="X107" t="n">
-        <v>25760.15</v>
+        <v>25762.04</v>
       </c>
     </row>
     <row r="108">
@@ -8949,7 +8949,7 @@
         <v>0</v>
       </c>
       <c r="X108" t="n">
-        <v>21509.11</v>
+        <v>21509.49</v>
       </c>
     </row>
     <row r="109">
@@ -9031,7 +9031,7 @@
         <v>0</v>
       </c>
       <c r="X109" t="n">
-        <v>122080.86</v>
+        <v>122248.85</v>
       </c>
     </row>
     <row r="110">
@@ -9113,7 +9113,7 @@
         <v>0</v>
       </c>
       <c r="X110" t="n">
-        <v>36779.88</v>
+        <v>36788</v>
       </c>
     </row>
     <row r="111">
@@ -9195,7 +9195,7 @@
         <v>0</v>
       </c>
       <c r="X111" t="n">
-        <v>85731.14</v>
+        <v>85895.86</v>
       </c>
     </row>
     <row r="112">
@@ -9275,7 +9275,7 @@
         <v>1</v>
       </c>
       <c r="X112" t="n">
-        <v>475131.17</v>
+        <v>472840.09</v>
       </c>
     </row>
     <row r="113">
@@ -9355,7 +9355,7 @@
         <v>0</v>
       </c>
       <c r="X113" t="n">
-        <v>318346.5</v>
+        <v>319280.72</v>
       </c>
     </row>
     <row r="114">
@@ -9437,7 +9437,7 @@
         <v>0</v>
       </c>
       <c r="X114" t="n">
-        <v>20483.95</v>
+        <v>20485.13</v>
       </c>
     </row>
     <row r="115">
@@ -9523,7 +9523,7 @@
         <v>0</v>
       </c>
       <c r="X115" t="n">
-        <v>171709.91</v>
+        <v>172414.79</v>
       </c>
     </row>
     <row r="116">
@@ -9603,7 +9603,7 @@
         <v>1</v>
       </c>
       <c r="X116" t="n">
-        <v>244288.16</v>
+        <v>243751.9</v>
       </c>
     </row>
     <row r="117">
@@ -9753,7 +9753,7 @@
         <v>1</v>
       </c>
       <c r="X118" t="n">
-        <v>310580.22</v>
+        <v>309606.56</v>
       </c>
     </row>
     <row r="119">
@@ -9833,7 +9833,7 @@
         <v>1</v>
       </c>
       <c r="X119" t="n">
-        <v>219429.27</v>
+        <v>218622.88</v>
       </c>
     </row>
     <row r="120">
@@ -9913,7 +9913,7 @@
         <v>0</v>
       </c>
       <c r="X120" t="n">
-        <v>207919.48</v>
+        <v>208710.18</v>
       </c>
     </row>
     <row r="121">
@@ -10065,7 +10065,7 @@
         <v>0</v>
       </c>
       <c r="X122" t="n">
-        <v>207534.75</v>
+        <v>207583.72</v>
       </c>
     </row>
     <row r="123">
@@ -10145,7 +10145,7 @@
         <v>0</v>
       </c>
       <c r="X123" t="n">
-        <v>385827.71</v>
+        <v>386974.85</v>
       </c>
     </row>
     <row r="124">
@@ -10435,7 +10435,7 @@
         <v>1</v>
       </c>
       <c r="X127" t="n">
-        <v>60534.81</v>
+        <v>60374.15</v>
       </c>
     </row>
     <row r="128">
@@ -10521,7 +10521,7 @@
         <v>0</v>
       </c>
       <c r="X128" t="n">
-        <v>45378.03</v>
+        <v>45650.83</v>
       </c>
     </row>
     <row r="129">
@@ -10607,7 +10607,7 @@
         <v>1</v>
       </c>
       <c r="X129" t="n">
-        <v>63797.97</v>
+        <v>63472.93</v>
       </c>
     </row>
     <row r="130">
@@ -10687,7 +10687,7 @@
         <v>0</v>
       </c>
       <c r="X130" t="n">
-        <v>56459.79</v>
+        <v>56703.7</v>
       </c>
     </row>
     <row r="131">
@@ -10767,7 +10767,7 @@
         <v>1</v>
       </c>
       <c r="X131" t="n">
-        <v>72350.58</v>
+        <v>72162.07000000001</v>
       </c>
     </row>
     <row r="132">
@@ -10849,7 +10849,7 @@
         <v>0</v>
       </c>
       <c r="X132" t="n">
-        <v>37826.77</v>
+        <v>37832.83</v>
       </c>
     </row>
     <row r="133">
@@ -10929,7 +10929,7 @@
         <v>1</v>
       </c>
       <c r="X133" t="n">
-        <v>53888.29</v>
+        <v>53628.05</v>
       </c>
     </row>
     <row r="134">
@@ -11079,7 +11079,7 @@
         <v>1</v>
       </c>
       <c r="X135" t="n">
-        <v>69719.66</v>
+        <v>69493.47</v>
       </c>
     </row>
     <row r="136">
@@ -11159,7 +11159,7 @@
         <v>1</v>
       </c>
       <c r="X136" t="n">
-        <v>85521.19</v>
+        <v>85072.14999999999</v>
       </c>
     </row>
     <row r="137">
@@ -11239,7 +11239,7 @@
         <v>1</v>
       </c>
       <c r="X137" t="n">
-        <v>61465.81</v>
+        <v>61236.77</v>
       </c>
     </row>
     <row r="138">
@@ -11319,7 +11319,7 @@
         <v>0</v>
       </c>
       <c r="X138" t="n">
-        <v>91909.87</v>
+        <v>92293.67999999999</v>
       </c>
     </row>
     <row r="139">
@@ -11471,7 +11471,7 @@
         <v>0</v>
       </c>
       <c r="X140" t="n">
-        <v>25079.7</v>
+        <v>25084.99</v>
       </c>
     </row>
     <row r="141">
@@ -11551,7 +11551,7 @@
         <v>1</v>
       </c>
       <c r="X141" t="n">
-        <v>54236.92</v>
+        <v>54071.68</v>
       </c>
     </row>
     <row r="142">
@@ -11637,7 +11637,7 @@
         <v>1</v>
       </c>
       <c r="X142" t="n">
-        <v>46665.99</v>
+        <v>46384.91</v>
       </c>
     </row>
     <row r="143">
@@ -11717,7 +11717,7 @@
         <v>0</v>
       </c>
       <c r="X143" t="n">
-        <v>81251.85000000001</v>
+        <v>81462.41</v>
       </c>
     </row>
     <row r="144">
@@ -11797,7 +11797,7 @@
         <v>1</v>
       </c>
       <c r="X144" t="n">
-        <v>43361.16</v>
+        <v>43225.31</v>
       </c>
     </row>
     <row r="145">
@@ -11953,7 +11953,7 @@
         <v>1</v>
       </c>
       <c r="X146" t="n">
-        <v>52215.68</v>
+        <v>51934.96</v>
       </c>
     </row>
     <row r="147">
@@ -12033,7 +12033,7 @@
         <v>1</v>
       </c>
       <c r="X147" t="n">
-        <v>56433.47</v>
+        <v>56175.01</v>
       </c>
     </row>
     <row r="148">
@@ -12113,7 +12113,7 @@
         <v>0</v>
       </c>
       <c r="X148" t="n">
-        <v>53176.12</v>
+        <v>53590.21</v>
       </c>
     </row>
     <row r="149">
@@ -12193,7 +12193,7 @@
         <v>0</v>
       </c>
       <c r="X149" t="n">
-        <v>48671.89</v>
+        <v>48973.13</v>
       </c>
     </row>
     <row r="150">
@@ -12273,7 +12273,7 @@
         <v>1</v>
       </c>
       <c r="X150" t="n">
-        <v>39249.53</v>
+        <v>39085.14</v>
       </c>
     </row>
     <row r="151">
@@ -12353,7 +12353,7 @@
         <v>1</v>
       </c>
       <c r="X151" t="n">
-        <v>35635.83</v>
+        <v>35471.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>